<commit_message>
adding floor_area_panel and integration in HP and Building model
</commit_message>
<xml_diff>
--- a/Results/data_centers_demand.xlsx
+++ b/Results/data_centers_demand.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ittuberlin-my.sharepoint.com/personal/17281442811011116638102512442_msopseudo_tu-berlin_de/Documents/Dokumente/2. WiIng/4. Masterarbeit SS26/Code/Results/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="483" documentId="13_ncr:1_{D3A18EBB-32A8-EA4D-8710-6AFC74E84898}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6AFC8D6B-377E-B74F-B8F0-51005F0E6B22}"/>
+  <xr:revisionPtr revIDLastSave="484" documentId="13_ncr:1_{D3A18EBB-32A8-EA4D-8710-6AFC74E84898}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DC5E7510-65F6-0E4B-B2C0-39AD7CB54F33}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Documentation" sheetId="4" r:id="rId1"/>
     <sheet name="ICIS" sheetId="1" r:id="rId2"/>
     <sheet name="Historical_2010_2024" sheetId="5" r:id="rId3"/>
-    <sheet name="ds_model_results" sheetId="2" r:id="rId4"/>
+    <sheet name="dc_model_results" sheetId="2" r:id="rId4"/>
     <sheet name="input_EnBW Model 2026" sheetId="3" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
@@ -795,13 +795,13 @@
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -7071,6 +7071,10 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -7364,40 +7368,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="33" t="s">
+      <c r="A1" s="34" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="33"/>
-      <c r="C1" s="33"/>
-      <c r="D1" s="33"/>
-      <c r="E1" s="33"/>
-      <c r="F1" s="33"/>
-      <c r="G1" s="33"/>
-      <c r="H1" s="33"/>
-      <c r="I1" s="33"/>
-      <c r="J1" s="33"/>
-      <c r="K1" s="33"/>
-      <c r="L1" s="33"/>
-      <c r="M1" s="33"/>
-      <c r="N1" s="33"/>
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
+      <c r="E1" s="34"/>
+      <c r="F1" s="34"/>
+      <c r="G1" s="34"/>
+      <c r="H1" s="34"/>
+      <c r="I1" s="34"/>
+      <c r="J1" s="34"/>
+      <c r="K1" s="34"/>
+      <c r="L1" s="34"/>
+      <c r="M1" s="34"/>
+      <c r="N1" s="34"/>
     </row>
     <row r="2" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="34" t="s">
+      <c r="A2" s="35" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="34"/>
-      <c r="C2" s="34"/>
-      <c r="D2" s="34"/>
-      <c r="E2" s="34"/>
-      <c r="F2" s="34"/>
-      <c r="G2" s="34"/>
-      <c r="H2" s="34"/>
-      <c r="I2" s="34"/>
-      <c r="J2" s="34"/>
-      <c r="K2" s="34"/>
-      <c r="L2" s="34"/>
-      <c r="M2" s="34"/>
-      <c r="N2" s="34"/>
+      <c r="B2" s="35"/>
+      <c r="C2" s="35"/>
+      <c r="D2" s="35"/>
+      <c r="E2" s="35"/>
+      <c r="F2" s="35"/>
+      <c r="G2" s="35"/>
+      <c r="H2" s="35"/>
+      <c r="I2" s="35"/>
+      <c r="J2" s="35"/>
+      <c r="K2" s="35"/>
+      <c r="L2" s="35"/>
+      <c r="M2" s="35"/>
+      <c r="N2" s="35"/>
     </row>
     <row r="3" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
@@ -10263,7 +10267,7 @@
       </c>
     </row>
     <row r="27" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A27" s="35" t="s">
+      <c r="A27" s="33" t="s">
         <v>33</v>
       </c>
       <c r="B27" s="32">

</xml_diff>